<commit_message>
Tilføj Filcolana Alva + hero-billeder til Alva og Tilia
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/yarns.xlsx
+++ b/content/yarns.xlsx
@@ -10,65 +10,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!A1:AC64</definedName>
   </definedNames>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Maskerummet Review</author>
-  </authors>
-  <commentList>
-    <comment ref="F20" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: sport
-Korrekt kategori er "lace" – Ravelry og producent angiver lace/fingering. Kilde: ravelry.com</t>
-      </text>
-    </comment>
-    <comment ref="I20" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: 5.0
-Korrekt min-pind er 3,5 mm (enkelt tråd 3,5–6 mm). Kilde: gepardgarn.dk</t>
-      </text>
-    </comment>
-    <comment ref="I45" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: 3.5
-Korrekt anbefalet pind er 6,0 mm (fast pind). Kilde: permin.dk / lindehobby.com</t>
-      </text>
-    </comment>
-    <comment ref="J45" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: 15.0
-Korrekt anbefalet pind er 6,0 mm. Værdien 15 er fejl. Kilde: permin.dk / lindehobby.com</t>
-      </text>
-    </comment>
-    <comment ref="I46" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: 3.5
-Korrekt anbefalet pind er 6,0 mm (fast pind). Kilde: lindehobby.com/permin-bella-color</t>
-      </text>
-    </comment>
-    <comment ref="J46" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: 15.0
-Korrekt anbefalet pind er 6,0 mm. Værdien 15 er fejl. Kilde: lindehobby.com/permin-bella-color</t>
-      </text>
-    </comment>
-    <comment ref="E50" authorId="0">
-      <text>
-        <t xml:space="preserve">⚠ MULIG FEJL
-Gemte værdi: Bomuld
-Korrekt fiber er 100% Lyocell (pailletter er 100% polyester). Kilde: woolwarehouse.co.uk / urbanyarns.com</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
@@ -460,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA65"/>
+  <dimension ref="A1:AA66"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -546,6 +487,9 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
       <c r="B2" t="str">
         <v>BC Garn</v>
       </c>
@@ -576,6 +520,24 @@
       <c r="K2">
         <v>25</v>
       </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
       <c r="R2" t="str">
         <v>handvask</v>
       </c>
@@ -590,6 +552,18 @@
       </c>
       <c r="V2" t="str">
         <v>["GOTS"]</v>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+      <c r="X2" t="str">
+        <v/>
+      </c>
+      <c r="Y2" t="str">
+        <v/>
+      </c>
+      <c r="Z2" t="str">
+        <v/>
       </c>
       <c r="AA2" t="str">
         <v>[{"fiber":"uld","percentage":55},{"fiber":"bomuld","percentage":45}]</v>
@@ -671,11 +645,17 @@
       <c r="Y3" t="str">
         <v>Luxor er et merceriseret bomuldsgarn i fingering-tykkelse (100% bomuld). Merceriseringen giver garnet en smuk glans, stærke og klare farver samt en meget tydelig maskedefinition. hBomulden stammer fra USA, mens garnet spindes og farves i Serbien. Farvestofferne er uden animalske ingredienser, så garnet kan betegnes som vegansk. Luxor kan maskinvaskes (op til 40 °C), men glansen kan aftage en smule over tid.</v>
       </c>
+      <c r="Z3" t="str">
+        <v/>
+      </c>
       <c r="AA3" t="str">
         <v>[{"fiber":"merceriseret_bomuld","percentage":100}]</v>
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
       <c r="B4" t="str">
         <v>BC Garn</v>
       </c>
@@ -706,6 +686,24 @@
       <c r="K4">
         <v>16</v>
       </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
       <c r="R4" t="str">
         <v>maskinvask_30</v>
       </c>
@@ -721,17 +719,35 @@
       <c r="V4" t="str">
         <v>["GOTS"]</v>
       </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+      <c r="Z4" t="str">
+        <v/>
+      </c>
       <c r="AA4" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
       <c r="B5" t="str">
         <v>Drops</v>
       </c>
       <c r="C5" t="str">
         <v>Air</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
       <c r="E5" t="str">
         <v>alpaka/uld/nylon</v>
       </c>
@@ -756,9 +772,15 @@
       <c r="L5">
         <v>22</v>
       </c>
+      <c r="M5" t="str">
+        <v/>
+      </c>
       <c r="N5" t="str">
         <v>Chainette/blown — fibre blæst ind i en tynd nylon-tube i stedet for klassisk spinding</v>
       </c>
+      <c r="O5" t="str">
+        <v/>
+      </c>
       <c r="P5" t="str">
         <v>chainette</v>
       </c>
@@ -788,6 +810,9 @@
       </c>
       <c r="Y5" t="str">
         <v>Lofty "blown" garn hvor baby-alpaka og merinould blæses ind i en tynd nylon-tube i stedet for at blive spundet. Færdige plagg er 30-35% lettere end tilsvarende tykkelse i klassisk spundet garn. Meget populær til behagelige oversize sweatre.</v>
+      </c>
+      <c r="Z5" t="str">
+        <v/>
       </c>
       <c r="AA5" t="str">
         <v>[{"fiber":"baby_alpaka","percentage":65},{"fiber":"nylon_polyamid","percentage":28},{"fiber":"merinould","percentage":7}]</v>
@@ -803,6 +828,9 @@
       <c r="C6" t="str">
         <v>Alaska</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
       <c r="E6" t="str">
         <v>Uld</v>
       </c>
@@ -848,6 +876,9 @@
       <c r="S6" t="str">
         <v>Norge</v>
       </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
       <c r="U6" t="str">
         <v>i_produktion</v>
       </c>
@@ -862,6 +893,9 @@
       </c>
       <c r="Y6" t="str">
         <v>Billigt budget-garn. Kan filtes.</v>
+      </c>
+      <c r="Z6" t="str">
+        <v/>
       </c>
       <c r="AA6" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -877,6 +911,9 @@
       <c r="C7" t="str">
         <v>Alpaca</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
       <c r="E7" t="str">
         <v>Alpaka</v>
       </c>
@@ -939,6 +976,9 @@
       </c>
       <c r="Y7" t="str">
         <v>Klassisk, let alpakagarn med fantastisk drapering og farvemætning. Populært til sjaler og lette projekter. Kradser ikke og er blødt mod huden. Et af DROPS' ældste og mest elskede kvaliteter.</v>
+      </c>
+      <c r="Z7" t="str">
+        <v/>
       </c>
       <c r="AA7" t="str">
         <v>[{"fiber":"alpaka","percentage":100}]</v>
@@ -954,6 +994,9 @@
       <c r="C8" t="str">
         <v>Brushed Alpaca Silk</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
       <c r="E8" t="str">
         <v>Alpaka-blanding</v>
       </c>
@@ -984,6 +1027,9 @@
       <c r="N8" t="str">
         <v>Brushed single, børstet superfin alpaka med silkekerne, kraftig halo</v>
       </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
       <c r="P8" t="str">
         <v>brushed_singles</v>
       </c>
@@ -996,6 +1042,9 @@
       <c r="S8" t="str">
         <v>Peru</v>
       </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
       <c r="U8" t="str">
         <v>i_produktion</v>
       </c>
@@ -1019,12 +1068,18 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
       <c r="B9" t="str">
         <v>Drops</v>
       </c>
       <c r="C9" t="str">
         <v>Flora</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
       <c r="E9" t="str">
         <v>uld/alpaka</v>
       </c>
@@ -1049,6 +1104,9 @@
       <c r="L9">
         <v>32</v>
       </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
       <c r="N9" t="str">
         <v>4-trådet plied fingering, uld + superfin alpaka, medium twist</v>
       </c>
@@ -1084,6 +1142,9 @@
       </c>
       <c r="Y9" t="str">
         <v>Slidstærkt fingering-garn med alpaka-blanding — særligt populær til sokker pga. holdbarheden. Tynd nok til colorwork og sjaler, blød nok til barnetøj.</v>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
       </c>
       <c r="AA9" t="str">
         <v>[{"fiber":"uld","percentage":65},{"fiber":"alpaka","percentage":35}]</v>
@@ -1099,6 +1160,9 @@
       <c r="C10" t="str">
         <v>Karisma</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
       <c r="E10" t="str">
         <v>Uld</v>
       </c>
@@ -1161,6 +1225,9 @@
       </c>
       <c r="Y10" t="str">
         <v>En af de absolut mest populære DROPS-kvaliteter. Slidstærkt, superwash-behandlet uldgarn til en meget prisvenlig pris. Fast twist giver god maskedefinition — god til farvemønstre.</v>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
       </c>
       <c r="AA10" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -1176,6 +1243,9 @@
       <c r="C11" t="str">
         <v>Merino Extra Fine</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
       <c r="E11" t="str">
         <v>Merinould</v>
       </c>
@@ -1238,6 +1308,9 @@
       </c>
       <c r="Y11" t="str">
         <v>Det foretrukne DK-garn fra DROPS — alsidigt, blødt og maskinvaskbart. Et af DROPS' absolut bedst sælgende garner i Danmark. Stor farvepalette og skarp pris.</v>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
       </c>
       <c r="AA11" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -1253,6 +1326,9 @@
       <c r="C12" t="str">
         <v>Safran</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
       <c r="E12" t="str">
         <v>Bomuld</v>
       </c>
@@ -1315,6 +1391,9 @@
       </c>
       <c r="Y12" t="str">
         <v>Go-to bomuldsgarn til sommerstrik og karklude. Enorm farvepalette og skarp pris — under 25 kr per nøgle. OEKO-TEX certificeret. Maskinvask 40°C på skåneprogram.</v>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
       </c>
       <c r="AA12" t="str">
         <v>[{"fiber":"bomuld","percentage":100}]</v>
@@ -1330,6 +1409,9 @@
       <c r="C13" t="str">
         <v>Wave</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
       <c r="E13" t="str">
         <v>Merinould-blanding</v>
       </c>
@@ -1360,6 +1442,9 @@
       <c r="N13" t="str">
         <v>Plied merino-silke-blanding, medium twist, blød og let glansfuld pga. silken</v>
       </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
       <c r="P13" t="str">
         <v>plied</v>
       </c>
@@ -1372,6 +1457,9 @@
       <c r="S13" t="str">
         <v>Italien</v>
       </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
       <c r="U13" t="str">
         <v>i_produktion</v>
       </c>
@@ -1387,17 +1475,26 @@
       <c r="Y13" t="str">
         <v>Specialgarn — ikke bredt distribueret i Danmark.</v>
       </c>
+      <c r="Z13" t="str">
+        <v/>
+      </c>
       <c r="AA13" t="str">
         <v>[{"fiber":"merinould","percentage":75},{"fiber":"silke","percentage":25}]</v>
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
       <c r="B14" t="str">
         <v>Filcolana</v>
       </c>
       <c r="C14" t="str">
         <v>Anina</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
       <c r="E14" t="str">
         <v>merino</v>
       </c>
@@ -1422,9 +1519,18 @@
       <c r="L14">
         <v>40</v>
       </c>
+      <c r="M14" t="str">
+        <v/>
+      </c>
+      <c r="N14" t="str">
+        <v/>
+      </c>
       <c r="O14">
         <v>4</v>
       </c>
+      <c r="P14" t="str">
+        <v/>
+      </c>
       <c r="Q14" t="str">
         <v>superwash</v>
       </c>
@@ -1434,8 +1540,26 @@
       <c r="S14" t="str">
         <v>Peru</v>
       </c>
+      <c r="T14" t="str">
+        <v/>
+      </c>
       <c r="U14" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V14" t="str">
+        <v/>
+      </c>
+      <c r="W14" t="str">
+        <v/>
+      </c>
+      <c r="X14" t="str">
+        <v/>
+      </c>
+      <c r="Y14" t="str">
+        <v/>
+      </c>
+      <c r="Z14" t="str">
+        <v/>
       </c>
       <c r="AA14" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -1451,6 +1575,9 @@
       <c r="C15" t="str">
         <v>Arwetta Classic</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
       <c r="E15" t="str">
         <v>Uld</v>
       </c>
@@ -1514,11 +1641,17 @@
       <c r="Y15" t="str">
         <v>Min go-to sokkegarn — slidstærk pga. nylon</v>
       </c>
+      <c r="Z15" t="str">
+        <v/>
+      </c>
       <c r="AA15" t="str">
         <v>[{"fiber":"merinould","percentage":80},{"fiber":"nylon_polyamid","percentage":20}]</v>
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
       <c r="B16" t="str">
         <v>Filcolana</v>
       </c>
@@ -1552,9 +1685,21 @@
       <c r="L16">
         <v>25</v>
       </c>
+      <c r="M16" t="str">
+        <v/>
+      </c>
+      <c r="N16" t="str">
+        <v/>
+      </c>
       <c r="O16">
         <v>4</v>
       </c>
+      <c r="P16" t="str">
+        <v/>
+      </c>
+      <c r="Q16" t="str">
+        <v/>
+      </c>
       <c r="R16" t="str">
         <v>handvask</v>
       </c>
@@ -1566,6 +1711,21 @@
       </c>
       <c r="U16" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V16" t="str">
+        <v/>
+      </c>
+      <c r="W16" t="str">
+        <v/>
+      </c>
+      <c r="X16" t="str">
+        <v/>
+      </c>
+      <c r="Y16" t="str">
+        <v/>
+      </c>
+      <c r="Z16" t="str">
+        <v/>
       </c>
       <c r="AA16" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -1581,6 +1741,9 @@
       <c r="C17" t="str">
         <v>Tilia</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
       <c r="E17" t="str">
         <v>Kid mohair</v>
       </c>
@@ -1610,6 +1773,9 @@
       </c>
       <c r="N17" t="str">
         <v>Brushed kid mohair single med silke, langfibret, kraftig halo</v>
+      </c>
+      <c r="O17" t="str">
+        <v/>
       </c>
       <c r="P17" t="str">
         <v>brushed_singles</v>
@@ -1643,6 +1809,9 @@
 _x000d__x000d_
 Kombinationen af silke og en let sky af mohair giver et luftigt, blødt og elegant udtryk – og er noget af det mest luksuriøse garn, man kan ønske sig at strikke med, både alene og som følgetråd.</v>
       </c>
+      <c r="Z17" t="str">
+        <v>/garn-eksempler/filcolana-tilia.jpg</v>
+      </c>
       <c r="AA17" t="str">
         <v>[{"fiber":"kid_mohair","percentage":70},{"fiber":"silke","percentage":30}]</v>
       </c>
@@ -1657,6 +1826,9 @@
       <c r="C18" t="str">
         <v>Ombelle</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
       <c r="E18" t="str">
         <v>Kid mohair-blanding</v>
       </c>
@@ -1687,6 +1859,9 @@
       <c r="N18" t="str">
         <v>Brushed mohair-blanding, single ply med langt halo</v>
       </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
       <c r="P18" t="str">
         <v>brushed_singles</v>
       </c>
@@ -1699,6 +1874,9 @@
       <c r="S18" t="str">
         <v>Frankrig</v>
       </c>
+      <c r="T18" t="str">
+        <v/>
+      </c>
       <c r="U18" t="str">
         <v>i_produktion</v>
       </c>
@@ -1714,11 +1892,17 @@
       <c r="Y18" t="str">
         <v>Fransk mohair-klassiker. Samme fibersammensætning som Permin Bella, men strikkes på meget mindre pind — fin let kvalitet snarere end chunky.</v>
       </c>
+      <c r="Z18" t="str">
+        <v/>
+      </c>
       <c r="AA18" t="str">
         <v>[{"fiber":"kid_mohair","percentage":75},{"fiber":"uld","percentage":20},{"fiber":"nylon_polyamid","percentage":5}]</v>
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
       <c r="B19" t="str">
         <v>Gepard</v>
       </c>
@@ -1749,17 +1933,50 @@
       <c r="K19">
         <v>22</v>
       </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+      <c r="M19" t="str">
+        <v/>
+      </c>
+      <c r="N19" t="str">
+        <v/>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+      <c r="Q19" t="str">
+        <v/>
+      </c>
       <c r="R19" t="str">
         <v>maskinvask_30</v>
       </c>
       <c r="S19" t="str">
         <v>Italien</v>
       </c>
+      <c r="T19" t="str">
+        <v/>
+      </c>
       <c r="U19" t="str">
         <v>i_produktion</v>
       </c>
       <c r="V19" t="str">
         <v>["GOTS (bomuld)","Oeko-Tex 100"]</v>
+      </c>
+      <c r="W19" t="str">
+        <v/>
+      </c>
+      <c r="X19" t="str">
+        <v/>
+      </c>
+      <c r="Y19" t="str">
+        <v/>
+      </c>
+      <c r="Z19" t="str">
+        <v/>
       </c>
       <c r="AA19" t="str">
         <v>[{"fiber":"bomuld","percentage":50},{"fiber":"merinould","percentage":50}]</v>
@@ -1775,6 +1992,9 @@
       <c r="C20" t="str">
         <v>Kid Silk 5</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
       <c r="E20" t="str">
         <v>Kid mohair</v>
       </c>
@@ -1805,6 +2025,9 @@
       <c r="N20" t="str">
         <v>Brushed single, kid mohair med silke, langfibret og kraftig halo</v>
       </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
       <c r="P20" t="str">
         <v>brushed_singles</v>
       </c>
@@ -1835,17 +2058,26 @@
       <c r="Y20" t="str">
         <v>Bliver løs i det med en tråd og dyr, hvis man skal strikke med 2 tråde</v>
       </c>
+      <c r="Z20" t="str">
+        <v/>
+      </c>
       <c r="AA20" t="str">
         <v>[{"fiber":"kid_mohair","percentage":80},{"fiber":"silke","percentage":20}]</v>
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
       <c r="B21" t="str">
         <v>Gepard</v>
       </c>
       <c r="C21" t="str">
         <v>Puno</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
       <c r="E21" t="str">
         <v>alpaka/merino/nylon</v>
       </c>
@@ -1867,14 +2099,50 @@
       <c r="K21">
         <v>12.5</v>
       </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+      <c r="M21" t="str">
+        <v/>
+      </c>
+      <c r="N21" t="str">
+        <v/>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+      <c r="Q21" t="str">
+        <v/>
+      </c>
       <c r="R21" t="str">
         <v>handvask</v>
       </c>
+      <c r="S21" t="str">
+        <v/>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
       <c r="U21" t="str">
         <v>i_produktion</v>
       </c>
       <c r="V21" t="str">
         <v>["RAS","RWS"]</v>
+      </c>
+      <c r="W21" t="str">
+        <v/>
+      </c>
+      <c r="X21" t="str">
+        <v/>
+      </c>
+      <c r="Y21" t="str">
+        <v/>
+      </c>
+      <c r="Z21" t="str">
+        <v/>
       </c>
       <c r="AA21" t="str">
         <v>[{"fiber":"baby_alpaka","percentage":68},{"fiber":"merinould","percentage":10},{"fiber":"nylon_polyamid","percentage":22}]</v>
@@ -1890,6 +2158,9 @@
       <c r="C22" t="str">
         <v>Extrafine Merino 90</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
       <c r="E22" t="str">
         <v>Merinould</v>
       </c>
@@ -1953,17 +2224,26 @@
       <c r="Y22" t="str">
         <v>Klassisk dansk storsælger fra Hjertegarn — bredt tilgængeligt i hele Danmark og meget prisvenligt. Superwash-behandlet merino i DK-tykkelse. Stor farvepalette og god kvalitet til hverdagsprojekter.</v>
       </c>
+      <c r="Z22" t="str">
+        <v/>
+      </c>
       <c r="AA22" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="str">
+        <v/>
+      </c>
       <c r="B23" t="str">
         <v>Holst Garn</v>
       </c>
       <c r="C23" t="str">
         <v>Coast</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
       <c r="E23" t="str">
         <v>uld/bomuld</v>
       </c>
@@ -1985,26 +2265,68 @@
       <c r="K23">
         <v>26</v>
       </c>
+      <c r="L23" t="str">
+        <v/>
+      </c>
+      <c r="M23" t="str">
+        <v/>
+      </c>
+      <c r="N23" t="str">
+        <v/>
+      </c>
       <c r="O23">
         <v>2</v>
       </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+      <c r="Q23" t="str">
+        <v/>
+      </c>
       <c r="R23" t="str">
         <v>maskinvask_30</v>
       </c>
+      <c r="S23" t="str">
+        <v/>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
       <c r="U23" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V23" t="str">
+        <v/>
+      </c>
+      <c r="W23" t="str">
+        <v/>
+      </c>
+      <c r="X23" t="str">
+        <v/>
+      </c>
+      <c r="Y23" t="str">
+        <v/>
+      </c>
+      <c r="Z23" t="str">
+        <v/>
       </c>
       <c r="AA23" t="str">
         <v>[{"fiber":"merinould","percentage":55},{"fiber":"bomuld","percentage":45}]</v>
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
       <c r="B24" t="str">
         <v>Holst Garn</v>
       </c>
       <c r="C24" t="str">
         <v>Supersoft</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
       <c r="E24" t="str">
         <v>merino/shetland</v>
       </c>
@@ -2026,14 +2348,50 @@
       <c r="K24">
         <v>25</v>
       </c>
+      <c r="L24" t="str">
+        <v/>
+      </c>
+      <c r="M24" t="str">
+        <v/>
+      </c>
+      <c r="N24" t="str">
+        <v/>
+      </c>
       <c r="O24">
         <v>2</v>
       </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+      <c r="Q24" t="str">
+        <v/>
+      </c>
       <c r="R24" t="str">
         <v>maskinvask_30</v>
       </c>
+      <c r="S24" t="str">
+        <v/>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
       <c r="U24" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V24" t="str">
+        <v/>
+      </c>
+      <c r="W24" t="str">
+        <v/>
+      </c>
+      <c r="X24" t="str">
+        <v/>
+      </c>
+      <c r="Y24" t="str">
+        <v/>
+      </c>
+      <c r="Z24" t="str">
+        <v/>
       </c>
       <c r="AA24" t="str">
         <v>[{"fiber":"merinould","percentage":50},{"fiber":"shetland_uld","percentage":50}]</v>
@@ -2049,6 +2407,9 @@
       <c r="C25" t="str">
         <v>Alpaca 2</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
       <c r="E25" t="str">
         <v>Alpaka-blanding</v>
       </c>
@@ -2112,17 +2473,26 @@
       <c r="Y25" t="str">
         <v>Isagers mest populære garn og en dansk klassiker siden 1977. Blød alpaka-uldblanding med smuk farvepalet og god drapering. Ikke-superwash — bæredygtig og holdbar. Meget brugt i Isager og Helga Isager opskrifter.</v>
       </c>
+      <c r="Z25" t="str">
+        <v/>
+      </c>
       <c r="AA25" t="str">
         <v>[{"fiber":"alpaka","percentage":50},{"fiber":"uld","percentage":50}]</v>
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
       <c r="B26" t="str">
         <v>Isager</v>
       </c>
       <c r="C26" t="str">
         <v>Jensen Yarn</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
       <c r="E26" t="str">
         <v>uld</v>
       </c>
@@ -2150,9 +2520,18 @@
       <c r="M26">
         <v>3</v>
       </c>
+      <c r="N26" t="str">
+        <v/>
+      </c>
       <c r="O26">
         <v>3</v>
       </c>
+      <c r="P26" t="str">
+        <v/>
+      </c>
+      <c r="Q26" t="str">
+        <v/>
+      </c>
       <c r="R26" t="str">
         <v>handvask</v>
       </c>
@@ -2165,17 +2544,38 @@
       <c r="U26" t="str">
         <v>i_produktion</v>
       </c>
+      <c r="V26" t="str">
+        <v/>
+      </c>
+      <c r="W26" t="str">
+        <v/>
+      </c>
+      <c r="X26" t="str">
+        <v/>
+      </c>
+      <c r="Y26" t="str">
+        <v/>
+      </c>
+      <c r="Z26" t="str">
+        <v/>
+      </c>
       <c r="AA26" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
       <c r="B27" t="str">
         <v>Isager</v>
       </c>
       <c r="C27" t="str">
         <v>Silk Mohair</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
       <c r="E27" t="str">
         <v>mohair/silke</v>
       </c>
@@ -2203,6 +2603,18 @@
       <c r="M27">
         <v>5</v>
       </c>
+      <c r="N27" t="str">
+        <v/>
+      </c>
+      <c r="O27" t="str">
+        <v/>
+      </c>
+      <c r="P27" t="str">
+        <v/>
+      </c>
+      <c r="Q27" t="str">
+        <v/>
+      </c>
       <c r="R27" t="str">
         <v>handvask</v>
       </c>
@@ -2217,6 +2629,18 @@
       </c>
       <c r="V27" t="str">
         <v>["RMS"]</v>
+      </c>
+      <c r="W27" t="str">
+        <v/>
+      </c>
+      <c r="X27" t="str">
+        <v/>
+      </c>
+      <c r="Y27" t="str">
+        <v/>
+      </c>
+      <c r="Z27" t="str">
+        <v/>
       </c>
       <c r="AA27" t="str">
         <v>[{"fiber":"kid_mohair","percentage":75},{"fiber":"silke","percentage":25}]</v>
@@ -2265,6 +2689,9 @@
       <c r="N28" t="str">
         <v>Let twistet, kraftigt woolen-spun, to tråde løst snoet</v>
       </c>
+      <c r="O28" t="str">
+        <v/>
+      </c>
       <c r="P28" t="str">
         <v>plied</v>
       </c>
@@ -2294,6 +2721,9 @@
       </c>
       <c r="Y28" t="str">
         <v>Den klassiske lopapeysa-tykkelse. Kradser på bar hud, men blødgøres ved vask. Varm og vandafvisende.</v>
+      </c>
+      <c r="Z28" t="str">
+        <v/>
       </c>
       <c r="AA28" t="str">
         <v>[{"fiber":"islandsk_uld","percentage":100}]</v>
@@ -2375,6 +2805,9 @@
       <c r="Y29" t="str">
         <v>Singles-garn med karakteristisk islandsk tovhet. God til sjaler og som holdtråd.</v>
       </c>
+      <c r="Z29" t="str">
+        <v/>
+      </c>
       <c r="AA29" t="str">
         <v>[{"fiber":"islandsk_uld","percentage":100}]</v>
       </c>
@@ -2455,6 +2888,9 @@
       <c r="Y30" t="str">
         <v>Light-version af Álafosslopi — halv vægt, halv tykkelse. Mest populære Lopi-kvalitet til moderne lopapeysa.</v>
       </c>
+      <c r="Z30" t="str">
+        <v/>
+      </c>
       <c r="AA30" t="str">
         <v>[{"fiber":"islandsk_uld","percentage":100}]</v>
       </c>
@@ -2502,6 +2938,9 @@
       <c r="N31" t="str">
         <v>Uspundet plate — skrøbelig tråd, skal håndteres varsomt</v>
       </c>
+      <c r="O31" t="str">
+        <v/>
+      </c>
       <c r="P31" t="str">
         <v>unspun</v>
       </c>
@@ -2532,17 +2971,26 @@
       <c r="Y31" t="str">
         <v>Kommer i runde plader à ca. 100 g. Kan holdes 2-3 tråde sammen for tykkere strik.</v>
       </c>
+      <c r="Z31" t="str">
+        <v/>
+      </c>
       <c r="AA31" t="str">
         <v>[{"fiber":"islandsk_uld","percentage":100}]</v>
       </c>
     </row>
     <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
       <c r="B32" t="str">
         <v>Knitting for Olive</v>
       </c>
       <c r="C32" t="str">
         <v>Cotton Merino</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
       <c r="E32" t="str">
         <v>bomuld/merino</v>
       </c>
@@ -2570,26 +3018,62 @@
       <c r="M32">
         <v>3</v>
       </c>
+      <c r="N32" t="str">
+        <v/>
+      </c>
+      <c r="O32" t="str">
+        <v/>
+      </c>
+      <c r="P32" t="str">
+        <v/>
+      </c>
+      <c r="Q32" t="str">
+        <v/>
+      </c>
       <c r="R32" t="str">
         <v>handvask</v>
       </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v/>
+      </c>
       <c r="U32" t="str">
         <v>i_produktion</v>
       </c>
       <c r="V32" t="str">
         <v>["Oeko-Tex Standard 100 (Class 1)","RWS","OCS"]</v>
       </c>
+      <c r="W32" t="str">
+        <v/>
+      </c>
+      <c r="X32" t="str">
+        <v/>
+      </c>
+      <c r="Y32" t="str">
+        <v/>
+      </c>
+      <c r="Z32" t="str">
+        <v/>
+      </c>
       <c r="AA32" t="str">
         <v>[{"fiber":"bomuld","percentage":70},{"fiber":"merinould","percentage":30}]</v>
       </c>
     </row>
     <row r="33">
+      <c r="A33" t="str">
+        <v/>
+      </c>
       <c r="B33" t="str">
         <v>Knitting for Olive</v>
       </c>
       <c r="C33" t="str">
         <v>Heavy Merino</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
       <c r="E33" t="str">
         <v>merino</v>
       </c>
@@ -2614,6 +3098,21 @@
       <c r="L33">
         <v>26</v>
       </c>
+      <c r="M33" t="str">
+        <v/>
+      </c>
+      <c r="N33" t="str">
+        <v/>
+      </c>
+      <c r="O33" t="str">
+        <v/>
+      </c>
+      <c r="P33" t="str">
+        <v/>
+      </c>
+      <c r="Q33" t="str">
+        <v/>
+      </c>
       <c r="R33" t="str">
         <v>handvask</v>
       </c>
@@ -2628,6 +3127,18 @@
       </c>
       <c r="V33" t="str">
         <v>["Oeko-Tex Standard 100"]</v>
+      </c>
+      <c r="W33" t="str">
+        <v/>
+      </c>
+      <c r="X33" t="str">
+        <v/>
+      </c>
+      <c r="Y33" t="str">
+        <v/>
+      </c>
+      <c r="Z33" t="str">
+        <v/>
       </c>
       <c r="AA33" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -2643,6 +3154,9 @@
       <c r="C34" t="str">
         <v>Merino</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
       <c r="E34" t="str">
         <v>Merinould</v>
       </c>
@@ -2705,6 +3219,9 @@
       </c>
       <c r="Y34" t="str">
         <v>KFO's suverænt mest solgte garn og det mest profilerede bæredygtige garnmærke i Danmark. Non-superwash, mulesing-fri og OEKO-TEX certificeret. Smukt farvekort og meget brugt i baby- og børnestrik.</v>
+      </c>
+      <c r="Z34" t="str">
+        <v/>
       </c>
       <c r="AA34" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -2720,6 +3237,9 @@
       <c r="C35" t="str">
         <v>Pure Silk</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
       <c r="E35" t="str">
         <v>Silke</v>
       </c>
@@ -2741,12 +3261,18 @@
       <c r="K35">
         <v>28</v>
       </c>
+      <c r="L35" t="str">
+        <v/>
+      </c>
       <c r="M35">
         <v>3</v>
       </c>
       <c r="N35" t="str">
         <v>Plied bourrette silke, medium twist, lidt rustik med synlige fiberender, mat finish</v>
       </c>
+      <c r="O35" t="str">
+        <v/>
+      </c>
       <c r="P35" t="str">
         <v>plied</v>
       </c>
@@ -2756,6 +3282,12 @@
       <c r="R35" t="str">
         <v>handvask</v>
       </c>
+      <c r="S35" t="str">
+        <v/>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
       <c r="U35" t="str">
         <v>i_produktion</v>
       </c>
@@ -2771,17 +3303,26 @@
       <c r="Y35" t="str">
         <v>Temperaturregulerende. Bourette silke giver mat finish frem for klassisk silkeglans.</v>
       </c>
+      <c r="Z35" t="str">
+        <v/>
+      </c>
       <c r="AA35" t="str">
         <v>[{"fiber":"silke","percentage":100}]</v>
       </c>
     </row>
     <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
       <c r="B36" t="str">
         <v>Lana Grossa</v>
       </c>
       <c r="C36" t="str">
         <v>Cool Wool</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
       <c r="E36" t="str">
         <v>merino</v>
       </c>
@@ -2806,6 +3347,21 @@
       <c r="L36">
         <v>34</v>
       </c>
+      <c r="M36" t="str">
+        <v/>
+      </c>
+      <c r="N36" t="str">
+        <v/>
+      </c>
+      <c r="O36" t="str">
+        <v/>
+      </c>
+      <c r="P36" t="str">
+        <v/>
+      </c>
+      <c r="Q36" t="str">
+        <v/>
+      </c>
       <c r="R36" t="str">
         <v>maskinvask_30</v>
       </c>
@@ -2817,6 +3373,21 @@
       </c>
       <c r="U36" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V36" t="str">
+        <v/>
+      </c>
+      <c r="W36" t="str">
+        <v/>
+      </c>
+      <c r="X36" t="str">
+        <v/>
+      </c>
+      <c r="Y36" t="str">
+        <v/>
+      </c>
+      <c r="Z36" t="str">
+        <v/>
       </c>
       <c r="AA36" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -2832,6 +3403,9 @@
       <c r="C37" t="str">
         <v>Maglia</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
       <c r="E37" t="str">
         <v>Bomuld-blanding</v>
       </c>
@@ -2862,6 +3436,9 @@
       <c r="N37" t="str">
         <v>Bomuldsblanding med let polyester-stretch</v>
       </c>
+      <c r="O37" t="str">
+        <v/>
+      </c>
       <c r="P37" t="str">
         <v>plied</v>
       </c>
@@ -2874,6 +3451,9 @@
       <c r="S37" t="str">
         <v>Italien</v>
       </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
       <c r="U37" t="str">
         <v>i_produktion</v>
       </c>
@@ -2889,11 +3469,17 @@
       <c r="Y37" t="str">
         <v>Bomuldsbaseret Lana Grossa-kvalitet med lille polyester-andel for form og styrke.</v>
       </c>
+      <c r="Z37" t="str">
+        <v/>
+      </c>
       <c r="AA37" t="str">
         <v>[{"fiber":"bomuld","percentage":92},{"fiber":"polyester","percentage":8}]</v>
       </c>
     </row>
     <row r="38">
+      <c r="A38" t="str">
+        <v/>
+      </c>
       <c r="B38" t="str">
         <v>Lang Yarns</v>
       </c>
@@ -2927,29 +3513,65 @@
       <c r="L38">
         <v>41</v>
       </c>
+      <c r="M38" t="str">
+        <v/>
+      </c>
+      <c r="N38" t="str">
+        <v/>
+      </c>
+      <c r="O38" t="str">
+        <v/>
+      </c>
+      <c r="P38" t="str">
+        <v/>
+      </c>
       <c r="Q38" t="str">
         <v>superwash</v>
       </c>
       <c r="R38" t="str">
         <v>maskinvask_40</v>
       </c>
+      <c r="S38" t="str">
+        <v/>
+      </c>
       <c r="T38" t="str">
         <v>Chile (Patagonia)</v>
       </c>
       <c r="U38" t="str">
         <v>i_produktion</v>
       </c>
+      <c r="V38" t="str">
+        <v/>
+      </c>
+      <c r="W38" t="str">
+        <v/>
+      </c>
+      <c r="X38" t="str">
+        <v/>
+      </c>
+      <c r="Y38" t="str">
+        <v/>
+      </c>
+      <c r="Z38" t="str">
+        <v/>
+      </c>
       <c r="AA38" t="str">
         <v>[{"fiber":"uld","percentage":75},{"fiber":"nylon_polyamid","percentage":25}]</v>
       </c>
     </row>
     <row r="39">
+      <c r="A39" t="str">
+        <v/>
+      </c>
       <c r="B39" t="str">
         <v>Lang Yarns</v>
       </c>
       <c r="C39" t="str">
         <v>Mille Colori Baby</v>
       </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
       <c r="E39" t="str">
         <v>merino</v>
       </c>
@@ -2974,29 +3596,65 @@
       <c r="L39">
         <v>36</v>
       </c>
+      <c r="M39" t="str">
+        <v/>
+      </c>
+      <c r="N39" t="str">
+        <v/>
+      </c>
+      <c r="O39" t="str">
+        <v/>
+      </c>
+      <c r="P39" t="str">
+        <v/>
+      </c>
       <c r="Q39" t="str">
         <v>superwash</v>
       </c>
       <c r="R39" t="str">
         <v>maskinvask_40</v>
       </c>
+      <c r="S39" t="str">
+        <v/>
+      </c>
       <c r="T39" t="str">
         <v>Australien</v>
       </c>
       <c r="U39" t="str">
         <v>i_produktion</v>
       </c>
+      <c r="V39" t="str">
+        <v/>
+      </c>
+      <c r="W39" t="str">
+        <v/>
+      </c>
+      <c r="X39" t="str">
+        <v/>
+      </c>
+      <c r="Y39" t="str">
+        <v/>
+      </c>
+      <c r="Z39" t="str">
+        <v/>
+      </c>
       <c r="AA39" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
       </c>
     </row>
     <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
       <c r="B40" t="str">
         <v>Manos del Uruguay</v>
       </c>
       <c r="C40" t="str">
         <v>Alegria</v>
       </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
       <c r="E40" t="str">
         <v>merino/nylon</v>
       </c>
@@ -3018,26 +3676,68 @@
       <c r="K40">
         <v>29</v>
       </c>
+      <c r="L40" t="str">
+        <v/>
+      </c>
+      <c r="M40" t="str">
+        <v/>
+      </c>
+      <c r="N40" t="str">
+        <v/>
+      </c>
+      <c r="O40" t="str">
+        <v/>
+      </c>
+      <c r="P40" t="str">
+        <v/>
+      </c>
       <c r="Q40" t="str">
         <v>superwash</v>
       </c>
       <c r="R40" t="str">
         <v>maskinvask_40</v>
       </c>
+      <c r="S40" t="str">
+        <v/>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
       <c r="U40" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V40" t="str">
+        <v/>
+      </c>
+      <c r="W40" t="str">
+        <v/>
+      </c>
+      <c r="X40" t="str">
+        <v/>
+      </c>
+      <c r="Y40" t="str">
+        <v/>
+      </c>
+      <c r="Z40" t="str">
+        <v/>
       </c>
       <c r="AA40" t="str">
         <v>[{"fiber":"merinould","percentage":75},{"fiber":"nylon_polyamid","percentage":25}]</v>
       </c>
     </row>
     <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
       <c r="B41" t="str">
         <v>Manos del Uruguay</v>
       </c>
       <c r="C41" t="str">
         <v>Serena</v>
       </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
       <c r="E41" t="str">
         <v>alpaka/bomuld</v>
       </c>
@@ -3059,14 +3759,50 @@
       <c r="K41">
         <v>24</v>
       </c>
+      <c r="L41" t="str">
+        <v/>
+      </c>
+      <c r="M41" t="str">
+        <v/>
+      </c>
+      <c r="N41" t="str">
+        <v/>
+      </c>
+      <c r="O41" t="str">
+        <v/>
+      </c>
+      <c r="P41" t="str">
+        <v/>
+      </c>
+      <c r="Q41" t="str">
+        <v/>
+      </c>
       <c r="R41" t="str">
         <v>handvask</v>
       </c>
+      <c r="S41" t="str">
+        <v/>
+      </c>
       <c r="T41" t="str">
         <v>Peru (alpaka), bomuld: ukendt</v>
       </c>
       <c r="U41" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V41" t="str">
+        <v/>
+      </c>
+      <c r="W41" t="str">
+        <v/>
+      </c>
+      <c r="X41" t="str">
+        <v/>
+      </c>
+      <c r="Y41" t="str">
+        <v/>
+      </c>
+      <c r="Z41" t="str">
+        <v/>
       </c>
       <c r="AA41" t="str">
         <v>[{"fiber":"baby_alpaka","percentage":60},{"fiber":"bomuld","percentage":40}]</v>
@@ -3082,6 +3818,9 @@
       <c r="C42" t="str">
         <v>Easy Care Big</v>
       </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
       <c r="E42" t="str">
         <v>Merinould</v>
       </c>
@@ -3124,6 +3863,9 @@
       <c r="R42" t="str">
         <v>maskinvask_40</v>
       </c>
+      <c r="S42" t="str">
+        <v/>
+      </c>
       <c r="T42" t="str">
         <v>Sydamerika</v>
       </c>
@@ -3141,6 +3883,9 @@
       </c>
       <c r="Y42" t="str">
         <v>Superwash-behandlet — kan maskinvaskes og tumbles. Bloomer mindre end ubehandlet uld og kan strække over tid.</v>
+      </c>
+      <c r="Z42" t="str">
+        <v/>
       </c>
       <c r="AA42" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -3156,6 +3901,9 @@
       <c r="C43" t="str">
         <v>Nordia</v>
       </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
       <c r="E43" t="str">
         <v>Uld-blanding</v>
       </c>
@@ -3177,9 +3925,18 @@
       <c r="K43">
         <v>19</v>
       </c>
+      <c r="L43" t="str">
+        <v/>
+      </c>
       <c r="M43">
         <v>4</v>
       </c>
+      <c r="N43" t="str">
+        <v/>
+      </c>
+      <c r="O43" t="str">
+        <v/>
+      </c>
       <c r="P43" t="str">
         <v>plied</v>
       </c>
@@ -3189,6 +3946,12 @@
       <c r="R43" t="str">
         <v>maskinvask_30</v>
       </c>
+      <c r="S43" t="str">
+        <v/>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
       <c r="U43" t="str">
         <v>i_produktion</v>
       </c>
@@ -3200,6 +3963,12 @@
       </c>
       <c r="X43" t="str">
         <v>[]</v>
+      </c>
+      <c r="Y43" t="str">
+        <v/>
+      </c>
+      <c r="Z43" t="str">
+        <v/>
       </c>
       <c r="AA43" t="str">
         <v>[{"fiber":"uld","percentage":51},{"fiber":"acryl","percentage":34},{"fiber":"nylon_polyamid","percentage":15}]</v>
@@ -3215,6 +3984,9 @@
       <c r="C44" t="str">
         <v>Trio</v>
       </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
       <c r="E44" t="str">
         <v>Uld</v>
       </c>
@@ -3277,6 +4049,9 @@
       </c>
       <c r="Y44" t="str">
         <v>Ubehandlet færøsk uld. Filter hvis behandlet forkert.</v>
+      </c>
+      <c r="Z44" t="str">
+        <v/>
       </c>
       <c r="AA44" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -3325,12 +4100,24 @@
       <c r="N45" t="str">
         <v>Brushed mohair-blanding med langt halo</v>
       </c>
+      <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v/>
+      </c>
       <c r="Q45" t="str">
         <v>standard</v>
       </c>
       <c r="R45" t="str">
         <v>handvask</v>
       </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v/>
+      </c>
       <c r="U45" t="str">
         <v>i_produktion</v>
       </c>
@@ -3342,9 +4129,15 @@
       </c>
       <c r="X45" t="str">
         <v>[]</v>
+      </c>
+      <c r="Y45" t="str">
+        <v/>
       </c>
       <c r="Z45" t="str">
         <v>/garn-eksempler/permin-bella.jpg</v>
+      </c>
+      <c r="AA45" t="str">
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -3390,6 +4183,9 @@
       <c r="N46" t="str">
         <v>Brushed mohair-blanding med langt halo</v>
       </c>
+      <c r="O46" t="str">
+        <v/>
+      </c>
       <c r="P46" t="str">
         <v>brushed_singles</v>
       </c>
@@ -3401,6 +4197,9 @@
       </c>
       <c r="S46" t="str">
         <v>Italien</v>
+      </c>
+      <c r="T46" t="str">
+        <v/>
       </c>
       <c r="U46" t="str">
         <v>i_produktion</v>
@@ -3434,6 +4233,9 @@
       <c r="C47" t="str">
         <v>Hannah</v>
       </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
       <c r="E47" t="str">
         <v>Merinould-blanding</v>
       </c>
@@ -3464,6 +4266,9 @@
       <c r="N47" t="str">
         <v>Brushed, silkekerne med uld/cashmere spundet udenom — let halo</v>
       </c>
+      <c r="O47" t="str">
+        <v/>
+      </c>
       <c r="P47" t="str">
         <v>brushed_singles</v>
       </c>
@@ -3476,6 +4281,9 @@
       <c r="S47" t="str">
         <v>Italien</v>
       </c>
+      <c r="T47" t="str">
+        <v/>
+      </c>
       <c r="U47" t="str">
         <v>i_produktion</v>
       </c>
@@ -3499,12 +4307,18 @@
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="str">
+        <v/>
+      </c>
       <c r="B48" t="str">
         <v>Rauma Garn</v>
       </c>
       <c r="C48" t="str">
         <v>Finull</v>
       </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
       <c r="E48" t="str">
         <v>uld</v>
       </c>
@@ -3526,9 +4340,24 @@
       <c r="K48">
         <v>25</v>
       </c>
+      <c r="L48" t="str">
+        <v/>
+      </c>
+      <c r="M48" t="str">
+        <v/>
+      </c>
+      <c r="N48" t="str">
+        <v/>
+      </c>
       <c r="O48">
         <v>2</v>
       </c>
+      <c r="P48" t="str">
+        <v/>
+      </c>
+      <c r="Q48" t="str">
+        <v/>
+      </c>
       <c r="R48" t="str">
         <v>maskinvask_30</v>
       </c>
@@ -3540,6 +4369,21 @@
       </c>
       <c r="U48" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V48" t="str">
+        <v/>
+      </c>
+      <c r="W48" t="str">
+        <v/>
+      </c>
+      <c r="X48" t="str">
+        <v/>
+      </c>
+      <c r="Y48" t="str">
+        <v/>
+      </c>
+      <c r="Z48" t="str">
+        <v/>
       </c>
       <c r="AA48" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -3555,6 +4399,9 @@
       <c r="C49" t="str">
         <v>Vams</v>
       </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
       <c r="E49" t="str">
         <v>Uld</v>
       </c>
@@ -3576,12 +4423,18 @@
       <c r="K49">
         <v>15</v>
       </c>
+      <c r="L49" t="str">
+        <v/>
+      </c>
       <c r="M49">
         <v>5.5</v>
       </c>
       <c r="N49" t="str">
         <v>Kardegarn (woolen-spun), single, blød twist, luftig og let filtbar</v>
       </c>
+      <c r="O49" t="str">
+        <v/>
+      </c>
       <c r="P49" t="str">
         <v>singles</v>
       </c>
@@ -3611,6 +4464,9 @@
       </c>
       <c r="Y49" t="str">
         <v>Kardegarn = kartet ulden er på kryds og tværs, hvilket giver et luftigt, blødt rustikt garn der bloomer kraftigt ved vask.</v>
+      </c>
+      <c r="Z49" t="str">
+        <v/>
       </c>
       <c r="AA49" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -3626,6 +4482,9 @@
       <c r="C50" t="str">
         <v>Creative Make It Blümchen</v>
       </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
       <c r="E50" t="str">
         <v>Lyocell</v>
       </c>
@@ -3638,9 +4497,30 @@
       <c r="H50">
         <v>1500</v>
       </c>
+      <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
+        <v/>
+      </c>
+      <c r="L50" t="str">
+        <v/>
+      </c>
+      <c r="M50" t="str">
+        <v/>
+      </c>
       <c r="N50" t="str">
         <v>Tråd med applikerede tekstil-blomster langs tråden (effektgarn)</v>
       </c>
+      <c r="O50" t="str">
+        <v/>
+      </c>
+      <c r="P50" t="str">
+        <v/>
+      </c>
       <c r="Q50" t="str">
         <v>standard</v>
       </c>
@@ -3650,6 +4530,9 @@
       <c r="S50" t="str">
         <v>Tyskland</v>
       </c>
+      <c r="T50" t="str">
+        <v/>
+      </c>
       <c r="U50" t="str">
         <v>i_produktion</v>
       </c>
@@ -3664,6 +4547,12 @@
       </c>
       <c r="Y50" t="str">
         <v>USIKKER — bekræft producent og specs på banderolen.</v>
+      </c>
+      <c r="Z50" t="str">
+        <v/>
+      </c>
+      <c r="AA50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -3676,6 +4565,9 @@
       <c r="C51" t="str">
         <v>Paillettes Classic Collection</v>
       </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
       <c r="E51" t="str">
         <v>Polyester</v>
       </c>
@@ -3697,9 +4589,21 @@
       <c r="K51">
         <v>28</v>
       </c>
+      <c r="L51" t="str">
+        <v/>
+      </c>
+      <c r="M51" t="str">
+        <v/>
+      </c>
       <c r="N51" t="str">
         <v>Tråd med indspundne/påsyede pailletter — effektgarn</v>
       </c>
+      <c r="O51" t="str">
+        <v/>
+      </c>
+      <c r="P51" t="str">
+        <v/>
+      </c>
       <c r="Q51" t="str">
         <v>standard</v>
       </c>
@@ -3709,6 +4613,9 @@
       <c r="S51" t="str">
         <v>Portugal</v>
       </c>
+      <c r="T51" t="str">
+        <v/>
+      </c>
       <c r="U51" t="str">
         <v>i_produktion</v>
       </c>
@@ -3723,6 +4630,12 @@
       </c>
       <c r="Y51" t="str">
         <v>USIKKER — Rosários 4 har flere pailletgarn-serier. Bør verificeres på banderolen.</v>
+      </c>
+      <c r="Z51" t="str">
+        <v/>
+      </c>
+      <c r="AA51" t="str">
+        <v/>
       </c>
     </row>
     <row r="52">
@@ -3735,6 +4648,9 @@
       <c r="C52" t="str">
         <v>Kitten Mohair</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
       <c r="E52" t="str">
         <v>Mohair-blanding</v>
       </c>
@@ -3765,6 +4681,9 @@
       <c r="N52" t="str">
         <v>Plied DK-mohair-blend, let halo, blødt</v>
       </c>
+      <c r="O52" t="str">
+        <v/>
+      </c>
       <c r="P52" t="str">
         <v>plied</v>
       </c>
@@ -3777,6 +4696,9 @@
       <c r="S52" t="str">
         <v>Norge</v>
       </c>
+      <c r="T52" t="str">
+        <v/>
+      </c>
       <c r="U52" t="str">
         <v>i_produktion</v>
       </c>
@@ -3792,17 +4714,26 @@
       <c r="Y52" t="str">
         <v>80er/90er-stilstrik. Akrylindholdet gør den mere robust og mindre elegant — ikke et luksusgarn til lette overdele.</v>
       </c>
+      <c r="Z52" t="str">
+        <v/>
+      </c>
       <c r="AA52" t="str">
         <v>[{"fiber":"courtelle","percentage":50},{"fiber":"mohair","percentage":30},{"fiber":"uld","percentage":20}]</v>
       </c>
     </row>
     <row r="53">
+      <c r="A53" t="str">
+        <v/>
+      </c>
       <c r="B53" t="str">
         <v>Sandnes Garn</v>
       </c>
       <c r="C53" t="str">
         <v>Kos</v>
       </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
       <c r="E53" t="str">
         <v>alpaka/uld/nylon</v>
       </c>
@@ -3824,26 +4755,68 @@
       <c r="K53">
         <v>17</v>
       </c>
+      <c r="L53" t="str">
+        <v/>
+      </c>
+      <c r="M53" t="str">
+        <v/>
+      </c>
+      <c r="N53" t="str">
+        <v/>
+      </c>
+      <c r="O53" t="str">
+        <v/>
+      </c>
+      <c r="P53" t="str">
+        <v/>
+      </c>
+      <c r="Q53" t="str">
+        <v/>
+      </c>
       <c r="R53" t="str">
         <v>maskinvask_30</v>
       </c>
+      <c r="S53" t="str">
+        <v/>
+      </c>
       <c r="T53" t="str">
         <v>Uruguay (uld), Peru (alpaka)</v>
       </c>
       <c r="U53" t="str">
         <v>i_produktion</v>
       </c>
+      <c r="V53" t="str">
+        <v/>
+      </c>
+      <c r="W53" t="str">
+        <v/>
+      </c>
+      <c r="X53" t="str">
+        <v/>
+      </c>
+      <c r="Y53" t="str">
+        <v/>
+      </c>
+      <c r="Z53" t="str">
+        <v/>
+      </c>
       <c r="AA53" t="str">
         <v>[{"fiber":"alpaka","percentage":62},{"fiber":"nylon_polyamid","percentage":29},{"fiber":"uld","percentage":9}]</v>
       </c>
     </row>
     <row r="54">
+      <c r="A54" t="str">
+        <v/>
+      </c>
       <c r="B54" t="str">
         <v>Sandnes Garn</v>
       </c>
       <c r="C54" t="str">
         <v>Line</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
       <c r="E54" t="str">
         <v>bomuld/viskose/lin</v>
       </c>
@@ -3865,14 +4838,50 @@
       <c r="K54">
         <v>20</v>
       </c>
+      <c r="L54" t="str">
+        <v/>
+      </c>
+      <c r="M54" t="str">
+        <v/>
+      </c>
+      <c r="N54" t="str">
+        <v/>
+      </c>
+      <c r="O54" t="str">
+        <v/>
+      </c>
+      <c r="P54" t="str">
+        <v/>
+      </c>
+      <c r="Q54" t="str">
+        <v/>
+      </c>
       <c r="R54" t="str">
         <v>maskinvask_30</v>
       </c>
+      <c r="S54" t="str">
+        <v/>
+      </c>
       <c r="T54" t="str">
         <v>Indien</v>
       </c>
       <c r="U54" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V54" t="str">
+        <v/>
+      </c>
+      <c r="W54" t="str">
+        <v/>
+      </c>
+      <c r="X54" t="str">
+        <v/>
+      </c>
+      <c r="Y54" t="str">
+        <v/>
+      </c>
+      <c r="Z54" t="str">
+        <v/>
       </c>
       <c r="AA54" t="str">
         <v>[{"fiber":"bomuld","percentage":53},{"fiber":"viskose","percentage":33},{"fiber":"lin","percentage":14}]</v>
@@ -3888,6 +4897,9 @@
       <c r="C55" t="str">
         <v>Peer Gynt</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
       <c r="E55" t="str">
         <v>Uld</v>
       </c>
@@ -3933,6 +4945,9 @@
       <c r="S55" t="str">
         <v>Norge</v>
       </c>
+      <c r="T55" t="str">
+        <v/>
+      </c>
       <c r="U55" t="str">
         <v>i_produktion</v>
       </c>
@@ -3947,6 +4962,9 @@
       </c>
       <c r="Y55" t="str">
         <v>Nordisk klassiker. Bredt farveudvalg. Meget brugt i PetiteKnit-opskrifter.</v>
+      </c>
+      <c r="Z55" t="str">
+        <v/>
       </c>
       <c r="AA55" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -3962,6 +4980,9 @@
       <c r="C56" t="str">
         <v>Poppy</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
       <c r="E56" t="str">
         <v>Bomuld</v>
       </c>
@@ -3992,6 +5013,9 @@
       <c r="N56" t="str">
         <v>Flertrådet, blød kæmmet bomuld</v>
       </c>
+      <c r="O56" t="str">
+        <v/>
+      </c>
       <c r="P56" t="str">
         <v>plied</v>
       </c>
@@ -4021,6 +5045,9 @@
       </c>
       <c r="Y56" t="str">
         <v>Blød bomuld uden glans, hverdagsprojekter i DK.</v>
+      </c>
+      <c r="Z56" t="str">
+        <v/>
       </c>
       <c r="AA56" t="str">
         <v>[{"fiber":"bomuld","percentage":100}]</v>
@@ -4036,6 +5063,9 @@
       <c r="C57" t="str">
         <v>Sunday</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
       <c r="E57" t="str">
         <v>Merinould</v>
       </c>
@@ -4098,6 +5128,9 @@
       </c>
       <c r="Y57" t="str">
         <v>Et af Sandnes' mest populære garner — ekstremt smukt farvekort med jordfarver og pasteller valgt i samarbejde med PetiteKnit. Non-superwash merino, meget blød. Bruges i mange af de mest downloadede opskrifter i Danmark.</v>
+      </c>
+      <c r="Z57" t="str">
+        <v/>
       </c>
       <c r="AA57" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -4113,6 +5146,9 @@
       <c r="C58" t="str">
         <v>Tynn Silk Mohair</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
       <c r="E58" t="str">
         <v>Kid mohair-blanding</v>
       </c>
@@ -4143,6 +5179,9 @@
       <c r="N58" t="str">
         <v>Brushed single, angora-ged mohair med silkekerne, medium halo</v>
       </c>
+      <c r="O58" t="str">
+        <v/>
+      </c>
       <c r="P58" t="str">
         <v>brushed_singles</v>
       </c>
@@ -4172,6 +5211,9 @@
       </c>
       <c r="Y58" t="str">
         <v>Meget populær silk mohair fra Sandnes — høj kvalitet, tåler maskinvask ved 30 grader (uldprogram), og bruges i mange gennemtestede opskrifter fra kendte strikkedesignere. Luksuriøs og luftig holdtråd.</v>
+      </c>
+      <c r="Z58" t="str">
+        <v/>
       </c>
       <c r="AA58" t="str">
         <v>[{"fiber":"mohair","percentage":57},{"fiber":"silke","percentage":28},{"fiber":"uld","percentage":15}]</v>
@@ -4235,6 +5277,9 @@
       <c r="S59" t="str">
         <v>Tyskland</v>
       </c>
+      <c r="T59" t="str">
+        <v/>
+      </c>
       <c r="U59" t="str">
         <v>i_produktion</v>
       </c>
@@ -4250,17 +5295,26 @@
       <c r="Y59" t="str">
         <v>Tysk sokkegarn-klassiker. Enormt farveudvalg inkl. selvstribende.</v>
       </c>
+      <c r="Z59" t="str">
+        <v/>
+      </c>
       <c r="AA59" t="str">
         <v>[{"fiber":"uld","percentage":75},{"fiber":"nylon_polyamid","percentage":25}]</v>
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="str">
+        <v/>
+      </c>
       <c r="B60" t="str">
         <v>Schoppel Wolle</v>
       </c>
       <c r="C60" t="str">
         <v>Edition 3</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
       <c r="E60" t="str">
         <v>merino</v>
       </c>
@@ -4279,26 +5333,71 @@
       <c r="J60">
         <v>3.5</v>
       </c>
+      <c r="K60" t="str">
+        <v/>
+      </c>
+      <c r="L60" t="str">
+        <v/>
+      </c>
+      <c r="M60" t="str">
+        <v/>
+      </c>
+      <c r="N60" t="str">
+        <v/>
+      </c>
+      <c r="O60" t="str">
+        <v/>
+      </c>
+      <c r="P60" t="str">
+        <v/>
+      </c>
       <c r="Q60" t="str">
         <v>superwash</v>
       </c>
       <c r="R60" t="str">
         <v>maskinvask_40</v>
       </c>
+      <c r="S60" t="str">
+        <v/>
+      </c>
+      <c r="T60" t="str">
+        <v/>
+      </c>
       <c r="U60" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V60" t="str">
+        <v/>
+      </c>
+      <c r="W60" t="str">
+        <v/>
+      </c>
+      <c r="X60" t="str">
+        <v/>
+      </c>
+      <c r="Y60" t="str">
+        <v/>
+      </c>
+      <c r="Z60" t="str">
+        <v/>
       </c>
       <c r="AA60" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
       </c>
     </row>
     <row r="61">
+      <c r="A61" t="str">
+        <v/>
+      </c>
       <c r="B61" t="str">
         <v>Schoppel Wolle</v>
       </c>
       <c r="C61" t="str">
         <v>Zauberball Stärke 6</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
       <c r="E61" t="str">
         <v>uld/nylon</v>
       </c>
@@ -4317,14 +5416,53 @@
       <c r="J61">
         <v>4</v>
       </c>
+      <c r="K61" t="str">
+        <v/>
+      </c>
+      <c r="L61" t="str">
+        <v/>
+      </c>
+      <c r="M61" t="str">
+        <v/>
+      </c>
+      <c r="N61" t="str">
+        <v/>
+      </c>
+      <c r="O61" t="str">
+        <v/>
+      </c>
+      <c r="P61" t="str">
+        <v/>
+      </c>
       <c r="Q61" t="str">
         <v>superwash</v>
       </c>
       <c r="R61" t="str">
         <v>maskinvask_40</v>
       </c>
+      <c r="S61" t="str">
+        <v/>
+      </c>
+      <c r="T61" t="str">
+        <v/>
+      </c>
       <c r="U61" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V61" t="str">
+        <v/>
+      </c>
+      <c r="W61" t="str">
+        <v/>
+      </c>
+      <c r="X61" t="str">
+        <v/>
+      </c>
+      <c r="Y61" t="str">
+        <v/>
+      </c>
+      <c r="Z61" t="str">
+        <v/>
       </c>
       <c r="AA61" t="str">
         <v>[{"fiber":"uld","percentage":75},{"fiber":"nylon_polyamid","percentage":25}]</v>
@@ -4340,6 +5478,9 @@
       <c r="C62" t="str">
         <v>Mohair Blend</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
       <c r="E62" t="str">
         <v>Kid mohair</v>
       </c>
@@ -4370,6 +5511,9 @@
       <c r="N62" t="str">
         <v>Brushed kid mohair single med syntetisk kerne, let halo</v>
       </c>
+      <c r="O62" t="str">
+        <v/>
+      </c>
       <c r="P62" t="str">
         <v>brushed_singles</v>
       </c>
@@ -4379,6 +5523,12 @@
       <c r="R62" t="str">
         <v>handvask</v>
       </c>
+      <c r="S62" t="str">
+        <v/>
+      </c>
+      <c r="T62" t="str">
+        <v/>
+      </c>
       <c r="U62" t="str">
         <v>i_produktion</v>
       </c>
@@ -4394,20 +5544,65 @@
       <c r="Y62" t="str">
         <v>Budget-alternativ til Tilia/Hannah. Mange bruger den til at teste mønstre før de investerer i dyrere mohair.</v>
       </c>
+      <c r="Z62" t="str">
+        <v/>
+      </c>
       <c r="AA62" t="str">
         <v>[{"fiber":"kid_mohair","percentage":80},{"fiber":"nylon_polyamid","percentage":20}]</v>
       </c>
     </row>
     <row r="63">
+      <c r="A63" t="str">
+        <v/>
+      </c>
       <c r="B63" t="str">
         <v>Tynd Uld / dansk spinderi</v>
       </c>
       <c r="C63" t="str">
         <v>Spelsau</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
       <c r="E63" t="str">
         <v>uld</v>
       </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+      <c r="H63" t="str">
+        <v/>
+      </c>
+      <c r="I63" t="str">
+        <v/>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
+        <v/>
+      </c>
+      <c r="L63" t="str">
+        <v/>
+      </c>
+      <c r="M63" t="str">
+        <v/>
+      </c>
+      <c r="N63" t="str">
+        <v/>
+      </c>
+      <c r="O63" t="str">
+        <v/>
+      </c>
+      <c r="P63" t="str">
+        <v/>
+      </c>
+      <c r="Q63" t="str">
+        <v/>
+      </c>
       <c r="R63" t="str">
         <v>ikke_angivet</v>
       </c>
@@ -4419,6 +5614,21 @@
       </c>
       <c r="U63" t="str">
         <v>i_produktion</v>
+      </c>
+      <c r="V63" t="str">
+        <v/>
+      </c>
+      <c r="W63" t="str">
+        <v/>
+      </c>
+      <c r="X63" t="str">
+        <v/>
+      </c>
+      <c r="Y63" t="str">
+        <v/>
+      </c>
+      <c r="Z63" t="str">
+        <v/>
       </c>
       <c r="AA63" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -4434,6 +5644,9 @@
       <c r="C64" t="str">
         <v>Korsika</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
       <c r="E64" t="str">
         <v>Plantefiber-blanding</v>
       </c>
@@ -4464,6 +5677,9 @@
       <c r="N64" t="str">
         <v>Plied plantefiber — mindre elasticitet end uld, falder tungt og pænt</v>
       </c>
+      <c r="O64" t="str">
+        <v/>
+      </c>
       <c r="P64" t="str">
         <v>plied</v>
       </c>
@@ -4476,6 +5692,9 @@
       <c r="S64" t="str">
         <v>Tyskland</v>
       </c>
+      <c r="T64" t="str">
+        <v/>
+      </c>
       <c r="U64" t="str">
         <v>i_produktion</v>
       </c>
@@ -4491,17 +5710,26 @@
       <c r="Y64" t="str">
         <v>Aldi-kampagnegarn. Kølig drape, ingen varme.</v>
       </c>
+      <c r="Z64" t="str">
+        <v/>
+      </c>
       <c r="AA64" t="str">
         <v>[{"fiber":"bomuld","percentage":73},{"fiber":"lin","percentage":27}]</v>
       </c>
     </row>
     <row r="65">
+      <c r="A65" t="str">
+        <v/>
+      </c>
       <c r="B65" t="str">
         <v>Drops</v>
       </c>
       <c r="C65" t="str">
         <v>Baby Merino</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
       <c r="E65" t="str">
         <v>merinould</v>
       </c>
@@ -4523,6 +5751,12 @@
       <c r="K65">
         <v>24</v>
       </c>
+      <c r="L65" t="str">
+        <v/>
+      </c>
+      <c r="M65" t="str">
+        <v/>
+      </c>
       <c r="N65" t="str">
         <v>3-trådet plied, superwash extrafine merino, medium twist</v>
       </c>
@@ -4566,13 +5800,93 @@
         <v>[{"fiber":"merinould","percentage":100}]</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v/>
+      </c>
+      <c r="B66" t="str">
+        <v>Filcolana</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Alva</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v>alpaka</v>
+      </c>
+      <c r="F66" t="str">
+        <v>lace</v>
+      </c>
+      <c r="G66">
+        <v>25</v>
+      </c>
+      <c r="H66">
+        <v>700</v>
+      </c>
+      <c r="I66" t="str">
+        <v/>
+      </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
+      <c r="K66" t="str">
+        <v/>
+      </c>
+      <c r="L66" t="str">
+        <v/>
+      </c>
+      <c r="M66" t="str">
+        <v/>
+      </c>
+      <c r="N66" t="str">
+        <v>tyndt 2-trådet alpakagarn</v>
+      </c>
+      <c r="O66">
+        <v>2</v>
+      </c>
+      <c r="P66" t="str">
+        <v>plied</v>
+      </c>
+      <c r="Q66" t="str">
+        <v/>
+      </c>
+      <c r="R66" t="str">
+        <v>handvask</v>
+      </c>
+      <c r="S66" t="str">
+        <v>Peru</v>
+      </c>
+      <c r="T66" t="str">
+        <v>Peru</v>
+      </c>
+      <c r="U66" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V66" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W66" t="str">
+        <v>[]</v>
+      </c>
+      <c r="X66" t="str">
+        <v>["følgegarn","sjaler","lette bluser"]</v>
+      </c>
+      <c r="Y66" t="str">
+        <v>Alva er et tyndt 2-trådet garn spundet af fibre fra peruvianske alpakaer. Alva er blød, varm og glansfuld og velegnet til mange slags projekter. Det tynde garn er perfekt til at strikke sammen med vores andre kvaliteter. Desuden er Alva et herligt alternativt følgegarn i stedet for et tyndt mohairgarn.</v>
+      </c>
+      <c r="Z66" t="str">
+        <v>/garn-eksempler/filcolana-alva.jpg</v>
+      </c>
+      <c r="AA66" t="str">
+        <v>[{"fiber":"alpaka","percentage":100}]</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AC64"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA65"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA66"/>
   </ignoredErrors>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Tilføj 13 garn-billeder + 8 nye Hjertegarn/Nordic Sky-garner
Hero-billeder til 5 eksisterende garner (Lana Grossa Cool Wool,
Lang Yarns Jawoll Superwash, BC Garn Bio Balance, BC Garn
Semilla Grosso, Hjertegarn Extrafine Merino 90) og 8 nye
garner: Hjertegarn Børstet Uld, Bamboo Wool, New Arezzo,
Alpaca 400, Dream Air, Brushed Armonia, Lima samt Nordic Sky
Kiruna.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/yarns.xlsx
+++ b/content/yarns.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AA100"/>
+  <dimension ref="A1:AA108"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -563,7 +563,7 @@
         <v/>
       </c>
       <c r="Z2" t="str">
-        <v/>
+        <v>/garn-eksempler/bc-garn-bio-balance.jpg</v>
       </c>
       <c r="AA2" t="str">
         <v>[{"fiber":"uld","percentage":55},{"fiber":"bomuld","percentage":45}]</v>
@@ -729,7 +729,7 @@
         <v/>
       </c>
       <c r="Z4" t="str">
-        <v/>
+        <v>/garn-eksempler/bc-garn-semilla-grosso.jpg</v>
       </c>
       <c r="AA4" t="str">
         <v>[{"fiber":"uld","percentage":100}]</v>
@@ -3387,7 +3387,7 @@
         <v>Klassisk dansk storsælger fra Hjertegarn — bredt tilgængeligt i hele Danmark og meget prisvenligt. Superwash-behandlet merino i DK-tykkelse. Stor farvepalette og god kvalitet til hverdagsprojekter.</v>
       </c>
       <c r="Z36" t="str">
-        <v/>
+        <v>/garn-eksempler/hjertegarn-extrafine-merino-90.jpg</v>
       </c>
       <c r="AA36" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -4798,7 +4798,7 @@
         <v/>
       </c>
       <c r="Z53" t="str">
-        <v/>
+        <v>/garn-eksempler/lana-grossa-cool-wool.jpg</v>
       </c>
       <c r="AA53" t="str">
         <v>[{"fiber":"merinould","percentage":100}]</v>
@@ -5047,7 +5047,7 @@
         <v/>
       </c>
       <c r="Z56" t="str">
-        <v/>
+        <v>/garn-eksempler/lang-yarns-jawoll-superwash.jpg</v>
       </c>
       <c r="AA56" t="str">
         <v>[{"fiber":"uld","percentage":75},{"fiber":"nylon_polyamid","percentage":25}]</v>
@@ -8705,9 +8705,673 @@
         <v>[{"fiber":"bomuld","percentage":53},{"fiber":"hør","percentage":47}]</v>
       </c>
     </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v/>
+      </c>
+      <c r="B101" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Børstet Uld</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v>uld/alpaka</v>
+      </c>
+      <c r="F101" t="str">
+        <v>bulky</v>
+      </c>
+      <c r="G101">
+        <v>50</v>
+      </c>
+      <c r="H101">
+        <v>300</v>
+      </c>
+      <c r="I101">
+        <v>7</v>
+      </c>
+      <c r="J101">
+        <v>8</v>
+      </c>
+      <c r="K101">
+        <v>14</v>
+      </c>
+      <c r="L101" t="str">
+        <v/>
+      </c>
+      <c r="M101">
+        <v>7</v>
+      </c>
+      <c r="N101" t="str">
+        <v/>
+      </c>
+      <c r="O101" t="str">
+        <v/>
+      </c>
+      <c r="P101" t="str">
+        <v>brushed_singles</v>
+      </c>
+      <c r="Q101" t="str">
+        <v>brushed</v>
+      </c>
+      <c r="R101" t="str">
+        <v>handvask</v>
+      </c>
+      <c r="S101" t="str">
+        <v/>
+      </c>
+      <c r="T101" t="str">
+        <v/>
+      </c>
+      <c r="U101" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V101" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W101" t="str">
+        <v>["vinter"]</v>
+      </c>
+      <c r="X101" t="str">
+        <v>["sweatre","jakker","huer","tørklæder","tæpper"]</v>
+      </c>
+      <c r="Y101" t="str">
+        <v>Børstet Uld fra Hjertegarn er et luftigt, lodden garn af 57% uld, 25% alpaka og 18% nylon. Den børstede overflade giver varme og volumen uden at gøre strikket tungt. Velegnet til hurtige projekter på pind 7-8 — sweatre, jakker og varme tilbehør.</v>
+      </c>
+      <c r="Z101" t="str">
+        <v>/garn-eksempler/hjertegarn-borstet-uld.jpg</v>
+      </c>
+      <c r="AA101" t="str">
+        <v>[{"fiber":"uld","percentage":57},{"fiber":"alpaka","percentage":25},{"fiber":"nylon_polyamid","percentage":18}]</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v/>
+      </c>
+      <c r="B102" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Bamboo Wool</v>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v>uld-blanding</v>
+      </c>
+      <c r="F102" t="str">
+        <v>fingering</v>
+      </c>
+      <c r="G102">
+        <v>50</v>
+      </c>
+      <c r="H102">
+        <v>400</v>
+      </c>
+      <c r="I102">
+        <v>2.5</v>
+      </c>
+      <c r="J102">
+        <v>3</v>
+      </c>
+      <c r="K102">
+        <v>28</v>
+      </c>
+      <c r="L102" t="str">
+        <v/>
+      </c>
+      <c r="M102">
+        <v>3</v>
+      </c>
+      <c r="N102" t="str">
+        <v/>
+      </c>
+      <c r="O102" t="str">
+        <v/>
+      </c>
+      <c r="P102" t="str">
+        <v>plied</v>
+      </c>
+      <c r="Q102" t="str">
+        <v>superwash</v>
+      </c>
+      <c r="R102" t="str">
+        <v>maskinvask_30</v>
+      </c>
+      <c r="S102" t="str">
+        <v/>
+      </c>
+      <c r="T102" t="str">
+        <v/>
+      </c>
+      <c r="U102" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V102" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W102" t="str">
+        <v>[]</v>
+      </c>
+      <c r="X102" t="str">
+        <v>["sokker","strømper","lette sweatre","babytøj"]</v>
+      </c>
+      <c r="Y102" t="str">
+        <v>Bamboo Wool fra Hjertegarn er et fingering-vægtet sok-/pulover-garn af 55% uld superwash, 30% bambus-viskose og 15% nylon. Bambusandelen giver et let, kølende skær og glat overflade, mens superwash-uld og nylon gør det slidstærkt — perfekt til sokker. Kan maskinvaskes ved uldprogram 30°.</v>
+      </c>
+      <c r="Z102" t="str">
+        <v>/garn-eksempler/hjertegarn-bamboo-wool.jpg</v>
+      </c>
+      <c r="AA102" t="str">
+        <v>[{"fiber":"uld","percentage":55},{"fiber":"viskose","percentage":30},{"fiber":"nylon_polyamid","percentage":15}]</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v/>
+      </c>
+      <c r="B103" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C103" t="str">
+        <v>New Arezzo</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v>plantefiber-blanding</v>
+      </c>
+      <c r="F103" t="str">
+        <v>sport</v>
+      </c>
+      <c r="G103">
+        <v>50</v>
+      </c>
+      <c r="H103">
+        <v>300</v>
+      </c>
+      <c r="I103">
+        <v>3</v>
+      </c>
+      <c r="J103">
+        <v>3.5</v>
+      </c>
+      <c r="K103">
+        <v>26</v>
+      </c>
+      <c r="L103" t="str">
+        <v/>
+      </c>
+      <c r="M103">
+        <v>3</v>
+      </c>
+      <c r="N103" t="str">
+        <v/>
+      </c>
+      <c r="O103" t="str">
+        <v/>
+      </c>
+      <c r="P103" t="str">
+        <v>plied</v>
+      </c>
+      <c r="Q103" t="str">
+        <v/>
+      </c>
+      <c r="R103" t="str">
+        <v>maskinvask_40</v>
+      </c>
+      <c r="S103" t="str">
+        <v/>
+      </c>
+      <c r="T103" t="str">
+        <v/>
+      </c>
+      <c r="U103" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V103" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W103" t="str">
+        <v>["sommer"]</v>
+      </c>
+      <c r="X103" t="str">
+        <v>["sommerbluser","tilbehør","lette projekter"]</v>
+      </c>
+      <c r="Y103" t="str">
+        <v>New Arezzo fra Hjertegarn er et plantegarn af 47% bambus-viskose, 33% hør og 20% bomuld. Bambus tilfører blødhed og glans, mens hør giver struktur og kølig drape — ideelt til sommerstrik som lette bluser og tilbehør. Strikkes på pind 3-3½ med ca. 26 masker pr. 10 cm.</v>
+      </c>
+      <c r="Z103" t="str">
+        <v>/garn-eksempler/hjertegarn-new-arezzo.jpg</v>
+      </c>
+      <c r="AA103" t="str">
+        <v>[{"fiber":"viskose","percentage":47},{"fiber":"hør","percentage":33},{"fiber":"bomuld","percentage":20}]</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v/>
+      </c>
+      <c r="B104" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C104" t="str">
+        <v>Alpaca 400</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v>alpaka</v>
+      </c>
+      <c r="F104" t="str">
+        <v>lace</v>
+      </c>
+      <c r="G104">
+        <v>50</v>
+      </c>
+      <c r="H104">
+        <v>800</v>
+      </c>
+      <c r="I104">
+        <v>2</v>
+      </c>
+      <c r="J104">
+        <v>3</v>
+      </c>
+      <c r="K104">
+        <v>30</v>
+      </c>
+      <c r="L104" t="str">
+        <v/>
+      </c>
+      <c r="M104">
+        <v>2.5</v>
+      </c>
+      <c r="N104" t="str">
+        <v/>
+      </c>
+      <c r="O104" t="str">
+        <v/>
+      </c>
+      <c r="P104" t="str">
+        <v>singles</v>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
+      </c>
+      <c r="R104" t="str">
+        <v>handvask</v>
+      </c>
+      <c r="S104" t="str">
+        <v/>
+      </c>
+      <c r="T104" t="str">
+        <v/>
+      </c>
+      <c r="U104" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V104" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W104" t="str">
+        <v>[]</v>
+      </c>
+      <c r="X104" t="str">
+        <v>["sjaler","tørklæder","blonder","følgegarn"]</v>
+      </c>
+      <c r="Y104" t="str">
+        <v>Alpaca 400 fra Hjertegarn er et tyndt lace-garn af 100% alpaka med 400 m pr. 50 g. Velegnet til sjaler og fine tørklæder, eller som følgegarn der gør tykkere garner blødere og lettere. Strikkes på pind 2-3 med ca. 30 masker pr. 10 cm. Håndvaskes.</v>
+      </c>
+      <c r="Z104" t="str">
+        <v>/garn-eksempler/hjertegarn-alpaca-400.jpg</v>
+      </c>
+      <c r="AA104" t="str">
+        <v>[{"fiber":"alpaka","percentage":100}]</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v/>
+      </c>
+      <c r="B105" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Dream Air</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v>uld/alpaka/nylon</v>
+      </c>
+      <c r="F105" t="str">
+        <v>bulky</v>
+      </c>
+      <c r="G105">
+        <v>50</v>
+      </c>
+      <c r="H105">
+        <v>400</v>
+      </c>
+      <c r="I105">
+        <v>6</v>
+      </c>
+      <c r="J105">
+        <v>6</v>
+      </c>
+      <c r="K105">
+        <v>17</v>
+      </c>
+      <c r="L105" t="str">
+        <v/>
+      </c>
+      <c r="M105">
+        <v>6</v>
+      </c>
+      <c r="N105" t="str">
+        <v/>
+      </c>
+      <c r="O105" t="str">
+        <v/>
+      </c>
+      <c r="P105" t="str">
+        <v>brushed_singles</v>
+      </c>
+      <c r="Q105" t="str">
+        <v>brushed</v>
+      </c>
+      <c r="R105" t="str">
+        <v>handvask</v>
+      </c>
+      <c r="S105" t="str">
+        <v/>
+      </c>
+      <c r="T105" t="str">
+        <v/>
+      </c>
+      <c r="U105" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V105" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W105" t="str">
+        <v>["vinter"]</v>
+      </c>
+      <c r="X105" t="str">
+        <v>["sweatre","cardigans","jakker","tæpper"]</v>
+      </c>
+      <c r="Y105" t="str">
+        <v>Dream Air fra Hjertegarn er et fabelagtigt blødt og luftigt børstet garn af 53% uld, 22% alpaka og 25% nylon. Trods tyngden strikker det op til en let og varm trøje — som at have luft på kroppen. Strikkes på pind 6 med ca. 17 masker pr. 10 cm. Håndvaskes.</v>
+      </c>
+      <c r="Z105" t="str">
+        <v>/garn-eksempler/hjertegarn-dream-air.jpg</v>
+      </c>
+      <c r="AA105" t="str">
+        <v>[{"fiber":"uld","percentage":53},{"fiber":"nylon_polyamid","percentage":25},{"fiber":"alpaka","percentage":22}]</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v/>
+      </c>
+      <c r="B106" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Brushed Armonia</v>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v>merino/nylon</v>
+      </c>
+      <c r="F106" t="str">
+        <v>fingering</v>
+      </c>
+      <c r="G106">
+        <v>50</v>
+      </c>
+      <c r="H106">
+        <v>400</v>
+      </c>
+      <c r="I106">
+        <v>3</v>
+      </c>
+      <c r="J106">
+        <v>4</v>
+      </c>
+      <c r="K106">
+        <v>28</v>
+      </c>
+      <c r="L106" t="str">
+        <v/>
+      </c>
+      <c r="M106">
+        <v>3</v>
+      </c>
+      <c r="N106" t="str">
+        <v/>
+      </c>
+      <c r="O106" t="str">
+        <v/>
+      </c>
+      <c r="P106" t="str">
+        <v>brushed_singles</v>
+      </c>
+      <c r="Q106" t="str">
+        <v>brushed</v>
+      </c>
+      <c r="R106" t="str">
+        <v>maskinvask_30</v>
+      </c>
+      <c r="S106" t="str">
+        <v/>
+      </c>
+      <c r="T106" t="str">
+        <v/>
+      </c>
+      <c r="U106" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V106" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W106" t="str">
+        <v>[]</v>
+      </c>
+      <c r="X106" t="str">
+        <v>["sweatre","cardigans","tilbehør","babytøj"]</v>
+      </c>
+      <c r="Y106" t="str">
+        <v>Brushed Armonia (Børstet Superfine Merino) fra Hjertegarn er et blødt, let børstet 4-trådet garn af 75% superwash merinould og 25% nylon. Børstningen giver et delikat halo, mens nylonet sikrer holdbarhed. Kan maskinvaskes ved uldprogram 30°. Strikkes på pind 3-4.</v>
+      </c>
+      <c r="Z106" t="str">
+        <v>/garn-eksempler/hjertegarn-brushed-armonia.jpg</v>
+      </c>
+      <c r="AA106" t="str">
+        <v>[{"fiber":"merinould","percentage":75},{"fiber":"nylon_polyamid","percentage":25}]</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v/>
+      </c>
+      <c r="B107" t="str">
+        <v>Hjertegarn</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Lima</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v>uld</v>
+      </c>
+      <c r="F107" t="str">
+        <v>worsted</v>
+      </c>
+      <c r="G107">
+        <v>50</v>
+      </c>
+      <c r="H107">
+        <v>200</v>
+      </c>
+      <c r="I107">
+        <v>4.5</v>
+      </c>
+      <c r="J107">
+        <v>5</v>
+      </c>
+      <c r="K107">
+        <v>20</v>
+      </c>
+      <c r="L107" t="str">
+        <v/>
+      </c>
+      <c r="M107">
+        <v>5</v>
+      </c>
+      <c r="N107" t="str">
+        <v/>
+      </c>
+      <c r="O107" t="str">
+        <v/>
+      </c>
+      <c r="P107" t="str">
+        <v>plied</v>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107" t="str">
+        <v>handvask</v>
+      </c>
+      <c r="S107" t="str">
+        <v/>
+      </c>
+      <c r="T107" t="str">
+        <v>Peru</v>
+      </c>
+      <c r="U107" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V107" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W107" t="str">
+        <v>[]</v>
+      </c>
+      <c r="X107" t="str">
+        <v>["sweatre","huer","vanter","tilbehør","filtning"]</v>
+      </c>
+      <c r="Y107" t="str">
+        <v>Lima fra Hjertegarn er et worsted-vægtet garn af 100% blød uld fra Peru. Garnet kradser mindre end mange tilsvarende kvaliteter og er velegnet til både børne- og voksenstrik. Kan filtes. Strikkes på pind 4½-5 med ca. 20 masker pr. 10 cm. Håndvaskes ved 30°.</v>
+      </c>
+      <c r="Z107" t="str">
+        <v>/garn-eksempler/hjertegarn-lima.jpg</v>
+      </c>
+      <c r="AA107" t="str">
+        <v>[{"fiber":"uld","percentage":100}]</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v/>
+      </c>
+      <c r="B108" t="str">
+        <v>Nordic Sky</v>
+      </c>
+      <c r="C108" t="str">
+        <v>Kiruna</v>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v>alpaka/merino/nylon</v>
+      </c>
+      <c r="F108" t="str">
+        <v>worsted</v>
+      </c>
+      <c r="G108">
+        <v>50</v>
+      </c>
+      <c r="H108">
+        <v>300</v>
+      </c>
+      <c r="I108">
+        <v>5</v>
+      </c>
+      <c r="J108">
+        <v>5</v>
+      </c>
+      <c r="K108">
+        <v>17</v>
+      </c>
+      <c r="L108">
+        <v>22</v>
+      </c>
+      <c r="M108">
+        <v>5</v>
+      </c>
+      <c r="N108" t="str">
+        <v/>
+      </c>
+      <c r="O108" t="str">
+        <v/>
+      </c>
+      <c r="P108" t="str">
+        <v>chainette</v>
+      </c>
+      <c r="Q108" t="str">
+        <v/>
+      </c>
+      <c r="R108" t="str">
+        <v>handvask</v>
+      </c>
+      <c r="S108" t="str">
+        <v>Sverige</v>
+      </c>
+      <c r="T108" t="str">
+        <v/>
+      </c>
+      <c r="U108" t="str">
+        <v>i_produktion</v>
+      </c>
+      <c r="V108" t="str">
+        <v>[]</v>
+      </c>
+      <c r="W108" t="str">
+        <v>[]</v>
+      </c>
+      <c r="X108" t="str">
+        <v>["sweatre","cardigans","huer","tørklæder"]</v>
+      </c>
+      <c r="Y108" t="str">
+        <v>Kiruna fra svenske Nordic Sky er et "blow yarn" af 63% baby-alpaka, 30% nylon og 7% merino. Fibrene blæses gennem et chainette-rør i stedet for at blive spundet på traditionel vis — det giver et meget let, blødt og volumiøst garn. Strikkes på pind 5 med 17 masker og 22 pinde pr. 10 cm. Håndvaskes ved 30°.</v>
+      </c>
+      <c r="Z108" t="str">
+        <v>/garn-eksempler/nordic-sky-kiruna.jpg</v>
+      </c>
+      <c r="AA108" t="str">
+        <v>[{"fiber":"baby_alpaka","percentage":63},{"fiber":"nylon_polyamid","percentage":30},{"fiber":"merinould","percentage":7}]</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AA100"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA108"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>